<commit_message>
testdata: prefix input columns with in_ in EligibilityDecision sheet
Aligns column names with SpecificContent key naming convention
so they match argument names in the decision workflows.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/Data/TestData/E2E.xlsx
+++ b/project/Data/TestData/E2E.xlsx
@@ -2,17 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="3348" windowWidth="30816" windowHeight="15852" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EligibilityDecision" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'EligibilityDecision'!$A$1:$M$36</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,8 +25,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -41,22 +40,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00264E8C"/>
+        <fgColor rgb="FF264E8C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFDDC1"/>
+        <fgColor rgb="FFFFDDC1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -69,10 +68,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -97,7 +105,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -461,15 +469,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M36"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="6" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
@@ -478,7 +485,7 @@
     <col width="52" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="29" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>TestCaseId</t>
@@ -491,42 +498,42 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CaseCategory</t>
+          <t>in_CaseCategory</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>ComplianceAssessment</t>
+          <t>in_ComplianceAssessment</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Attribute_A</t>
+          <t>in_Attribute_A</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Attribute_B</t>
+          <t>in_Attribute_B</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Attribute_C</t>
+          <t>in_Attribute_C</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Indicator_X</t>
+          <t>in_Indicator_X</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Detail_X</t>
+          <t>in_Detail_X</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>SecondaryIndicator</t>
+          <t>in_SecondaryIndicator</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -566,11 +573,11 @@
           <t>Compliant</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="b">
         <v>0</v>
       </c>
@@ -609,11 +616,11 @@
           <t>Compliant</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
       <c r="J3" s="2" t="b">
         <v>0</v>
       </c>
@@ -625,9 +632,9 @@
       <c r="L3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
+      <c r="M3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="29" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>RG1-P-003</t>
@@ -658,9 +665,9 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="b">
         <v>0</v>
       </c>
@@ -678,7 +685,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="29" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>RG1-P-004</t>
@@ -704,14 +711,14 @@
           <t>Verification_not_available</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="n"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="b">
         <v>0</v>
       </c>
@@ -729,7 +736,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>RG1-P-005</t>
@@ -765,8 +772,8 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="b">
         <v>0</v>
       </c>
@@ -784,7 +791,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>RG1-P-006</t>
@@ -815,9 +822,9 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="b">
         <v>0</v>
       </c>
@@ -829,9 +836,9 @@
       <c r="L7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
+      <c r="M7" s="2" t="n"/>
+    </row>
+    <row r="8" ht="29" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>RG1-P-007</t>
@@ -857,14 +864,14 @@
           <t>Special_case_without_certified_component</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="n"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="b">
         <v>0</v>
       </c>
@@ -876,7 +883,7 @@
       <c r="L8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -894,12 +901,12 @@
           <t>Event_A</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="b">
         <v>0</v>
       </c>
@@ -933,12 +940,12 @@
           <t>Event_B</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="b">
         <v>0</v>
       </c>
@@ -992,8 +999,8 @@
           <t>OtherImpact</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="b">
         <v>1</v>
       </c>
@@ -1037,10 +1044,10 @@
           <t>OtherAttribute</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="b">
         <v>1</v>
       </c>
@@ -1058,7 +1065,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="29" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>RG1-N-001</t>
@@ -1094,8 +1101,8 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
       <c r="J13" s="2" t="b">
         <v>0</v>
       </c>
@@ -1149,8 +1156,8 @@
           <t>OtherImpact</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="b">
         <v>0</v>
       </c>
@@ -1204,8 +1211,8 @@
           <t>OtherImpact</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="b">
         <v>0</v>
       </c>
@@ -1217,9 +1224,9 @@
       <c r="L15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="M15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
+      <c r="M15" s="2" t="n"/>
+    </row>
+    <row r="16" ht="29" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>RG1-OQ-001</t>
@@ -1255,8 +1262,8 @@
           <t>OtherImpact</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="b">
         <v>0</v>
       </c>
@@ -1274,7 +1281,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="29" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>RG1-OQ-002</t>
@@ -1310,8 +1317,8 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="b">
         <v>0</v>
       </c>
@@ -1345,10 +1352,10 @@
           <t>Event_C</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1370,7 +1377,7 @@
       <c r="L18" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1388,16 +1395,16 @@
           <t>Event_C</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="b">
         <v>0</v>
       </c>
@@ -1431,10 +1438,10 @@
           <t>Event_D</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1456,7 +1463,7 @@
       <c r="L20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1474,16 +1481,16 @@
           <t>Event_D</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="b">
         <v>0</v>
       </c>
@@ -1495,7 +1502,7 @@
       <c r="L21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1518,15 +1525,15 @@
           <t>Compliant</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="b">
         <v>0</v>
       </c>
@@ -1538,7 +1545,7 @@
       <c r="L22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1561,15 +1568,15 @@
           <t>Compliant</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="b">
         <v>0</v>
       </c>
@@ -1581,9 +1588,9 @@
       <c r="L23" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
+      <c r="M23" s="2" t="n"/>
+    </row>
+    <row r="24" ht="29" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>RG2-P-007</t>
@@ -1614,13 +1621,13 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="n"/>
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="b">
         <v>0</v>
       </c>
@@ -1632,9 +1639,9 @@
       <c r="L24" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
+      <c r="M24" s="2" t="n"/>
+    </row>
+    <row r="25" ht="29" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>RG2-P-008</t>
@@ -1660,7 +1667,7 @@
           <t>Verification_not_available</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="n"/>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>No_or_low_impact</t>
@@ -1671,7 +1678,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="n"/>
       <c r="J25" s="2" t="b">
         <v>0</v>
       </c>
@@ -1683,9 +1690,9 @@
       <c r="L25" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
+      <c r="M25" s="2" t="n"/>
+    </row>
+    <row r="26" ht="29" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>RG2-P-009</t>
@@ -1716,13 +1723,13 @@
           <t>No_or_low_impact</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="n"/>
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="n"/>
       <c r="J26" s="2" t="b">
         <v>0</v>
       </c>
@@ -1734,9 +1741,9 @@
       <c r="L26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
+      <c r="M26" s="2" t="n"/>
+    </row>
+    <row r="27" ht="29" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>RG2-P-010</t>
@@ -1762,7 +1769,7 @@
           <t>Special_case_without_certified_component</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="n"/>
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>No_or_low_impact</t>
@@ -1773,7 +1780,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="n"/>
       <c r="J27" s="2" t="b">
         <v>0</v>
       </c>
@@ -1785,7 +1792,7 @@
       <c r="L27" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1803,16 +1810,16 @@
           <t>Event_C</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="n"/>
       <c r="J28" s="2" t="b">
         <v>0</v>
       </c>
@@ -1830,7 +1837,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="29" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>RG2-P-012</t>
@@ -1846,16 +1853,16 @@
           <t>Event_D</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="n"/>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="n"/>
       <c r="J29" s="2" t="b">
         <v>0</v>
       </c>
@@ -1867,7 +1874,7 @@
       <c r="L29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1910,7 +1917,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="n"/>
       <c r="J30" s="2" t="b">
         <v>1</v>
       </c>
@@ -1954,14 +1961,14 @@
           <t>OtherAttribute</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="n"/>
       <c r="J31" s="2" t="b">
         <v>1</v>
       </c>
@@ -1973,9 +1980,9 @@
       <c r="L31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
+      <c r="M31" s="2" t="n"/>
+    </row>
+    <row r="32" ht="29" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>RG2-N-001</t>
@@ -2016,7 +2023,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="b">
         <v>0</v>
       </c>
@@ -2034,7 +2041,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="29" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>RG2-N-002</t>
@@ -2075,7 +2082,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="n"/>
       <c r="J33" s="2" t="b">
         <v>0</v>
       </c>
@@ -2087,9 +2094,9 @@
       <c r="L33" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
+      <c r="M33" s="2" t="n"/>
+    </row>
+    <row r="34" ht="29" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>RG2-N-003</t>
@@ -2130,7 +2137,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="n"/>
       <c r="J34" s="2" t="b">
         <v>0</v>
       </c>
@@ -2142,9 +2149,9 @@
       <c r="L34" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
+      <c r="M34" s="2" t="n"/>
+    </row>
+    <row r="35" ht="29" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>RG2-OQ-001</t>
@@ -2185,7 +2192,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="n"/>
       <c r="J35" s="2" t="b">
         <v>0</v>
       </c>
@@ -2203,7 +2210,7 @@
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="29" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>RG2-OQ-002</t>
@@ -2244,7 +2251,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="n"/>
       <c r="J36" s="2" t="b">
         <v>0</v>
       </c>
@@ -2263,7 +2270,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
annotations: add structured educational annotations to all workflows
Applies two-axis annotation scheme (structure + logic) to all 13 XAML
workflows across EligibilityDecision (5) and RoutingPipeline (8).

Each workflow has:
- A docked Sequence-level annotation with pattern, I/O, and structure summary
- Per-activity annotations explaining rules, expressions, sentinels, and patterns
- One needle (#cb39fe) marking the consequential decision activity

Also adds annotation plan YAMLs (_annotations_plan.yml) as source-of-truth
for the annotation content, and includes RoutingPipeline test data in E2E.xlsx.

Fix: IsExpanded must precede IsAnnotationDocked in ViewState Dictionary
when both keys are present on Sequence elements that have Sequence.Variables.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/Data/TestData/E2E.xlsx
+++ b/project/Data/TestData/E2E.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EligibilityDecision" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RoutingPipeline" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -2272,4 +2273,1138 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TestCaseId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>in_HasRegistryId</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>in_RegistryParticipantExists</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>in_DocumentTypesAccepted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>in_RegistryId</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>in_VatId</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>in_CustomerExists</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>in_IsSegmentP</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>in_HasCustomerErrors</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>in_HasInternalErrors</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Expected_RoutingDecision</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>RuleGroup</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RP-HP-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Channel_A, PS, NATIONAL, EXISTING, SegP=F</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PS-001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>DOM-123</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>RP-HP-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Channel_B (no HasRegistryId), non-PS, INTERNATIONAL, NEW, SegP=F</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>CORP-001</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>INT-456</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>RP-HP-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Channel_B (no Participant), PS, NATIONAL, EXISTING, SegP=T</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PS-002</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DOM-789</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Segment_P notification fires</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RP-HP-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Channel_B (no DocumentTypes), non-PS, INTERNATIONAL, NEW, SegP=F</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CORP-002</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>INT-999</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RP-HP-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Channel_A, non-PS, INTERNATIONAL, EXISTING, SegP=T</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CORP-003</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>INT-111</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>HAPPY_PATH</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RP-RC-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Channel_A, PS, NATIONAL, EXISTING, SegP=F</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PS-001</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DOM-123</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RP-RC-002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Channel_B (no HasRegistryId), non-PS, INTERNATIONAL, NEW, SegP=F</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CORP-001</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>INT-456</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RP-RC-003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Channel_A, PS, INTERNATIONAL, NEW, SegP=T</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PS-003</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>INT-222</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Segment_P with customer errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RP-RC-004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Channel_B (no Participant), non-PS, NATIONAL, EXISTING, SegP=F</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CORP-004</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DOM-333</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_CUSTOMER</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RP-RI-001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Channel_A, PS, NATIONAL, EXISTING, SegP=F</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PS-001</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DOM-123</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_INTERNAL</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RP-RI-002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Channel_B (no HasRegistryId), non-PS, INTERNATIONAL, NEW, SegP=F</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CORP-001</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>INT-456</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_INTERNAL</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RP-RI-003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Channel_A, non-PS, NATIONAL, NEW, SegP=T</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>CORP-005</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>DOM-444</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_INTERNAL</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Segment_P with internal errors</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RP-RI-004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Channel_B (no DocumentTypes), PS, INTERNATIONAL, EXISTING, SegP=F</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PS-004</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>INT-555</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>ROUTE_TO_INTERNAL</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RP-OQ-001</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Both errors — Channel_A, PS, NATIONAL, EXISTING</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PS-001</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>DOM-123</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>[OPEN] Precedence unresolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RP-OQ-002</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Both errors — Channel_B, non-PS, INTERNATIONAL, NEW</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>CORP-001</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>INT-456</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>[OPEN] Channel_B variant</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RP-OQ-003</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Both errors — Channel_A, non-PS, NATIONAL, NEW, SegP=T</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>CORP-006</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>DOM-666</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>[OPEN] With Segment_P notification</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>